<commit_message>
🐞 bug-fix: Resolving a bug or error preventing error on update_checker & salas.xlsx
</commit_message>
<xml_diff>
--- a/Planilhas/SALAS.xlsx
+++ b/Planilhas/SALAS.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sereducacionalbr-my.sharepoint.com/personal/dhiego_moura_sereducacional_com/Documents/Documentos/BB_Py_Automation-dev/BB_Py_Automation/Planilhas/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\013190873\Documents\VS\BB_Py_Automation\planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="11_A831CAF7196FC6FEBDF7265BE96BB01D44075CD0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D60E1653-6758-44EB-8E9A-40A82C818FF6}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE6121A9-B5FB-4A4B-9717-88F78B5D83CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1350" yWindow="1560" windowWidth="14730" windowHeight="11340" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="salas" sheetId="1" r:id="rId1"/>
@@ -385,7 +385,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -397,19 +397,10 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
@@ -728,137 +719,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:B114"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.5703125" style="9" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="17" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="19" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="22" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="30" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="32" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="33" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="48" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="49" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="50" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="51" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="52" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="53" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="54" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="55" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="56" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="57" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="58" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="59" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="60" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="61" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="62" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="63" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="64" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="65" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="66" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="67" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="68" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="69" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="70" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="71" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="72" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="73" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="74" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="75" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="76" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="77" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="78" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="79" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="80" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="81" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="82" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="83" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="84" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="85" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="86" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="87" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="88" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="89" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="90" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="91" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="92" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="93" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="94" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="95" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="96" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="97" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="98" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="99" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B99" s="1"/>
-    </row>
-    <row r="100" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="101" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="102" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="103" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="104" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="105" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="106" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="107" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="108" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="109" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="110" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="111" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="112" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="113" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="114" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B114" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -897,7 +771,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E8C6456-2450-485E-AC53-AFD9A36CC2D4}">
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.42578125" customWidth="1"/>
@@ -905,7 +779,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -914,189 +788,6 @@
       <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="8"/>
-      <c r="C2" s="3"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="7"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="7"/>
-      <c r="C4" s="5"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="7"/>
-      <c r="C5" s="5"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="7"/>
-      <c r="C6" s="5"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="7"/>
-      <c r="C7" s="5"/>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="7"/>
-      <c r="C8" s="5"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="7"/>
-      <c r="C9" s="5"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="7"/>
-      <c r="C10" s="5"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="7"/>
-      <c r="C11" s="5"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="7"/>
-      <c r="C12" s="5"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="7"/>
-      <c r="C13" s="5"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="7"/>
-      <c r="C14" s="5"/>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="7"/>
-      <c r="C15" s="5"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="7"/>
-      <c r="C16" s="5"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="7"/>
-      <c r="C17" s="5"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="7"/>
-      <c r="C18" s="5"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="7"/>
-      <c r="C19" s="5"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="7"/>
-      <c r="C20" s="5"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="7"/>
-      <c r="C21" s="5"/>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="7"/>
-      <c r="C22" s="5"/>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="7"/>
-      <c r="C23" s="5"/>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="7"/>
-      <c r="C24" s="5"/>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="7"/>
-      <c r="C25" s="5"/>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="7"/>
-      <c r="C26" s="5"/>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="7"/>
-      <c r="C27" s="5"/>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="7"/>
-      <c r="C28" s="5"/>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="7"/>
-      <c r="C29" s="5"/>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="7"/>
-      <c r="C30" s="5"/>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="7"/>
-      <c r="C31" s="5"/>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="7"/>
-      <c r="C32" s="5"/>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="7"/>
-      <c r="C33" s="5"/>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="7"/>
-      <c r="C34" s="5"/>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="7"/>
-      <c r="C35" s="6"/>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="7"/>
-      <c r="C36" s="5"/>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="7"/>
-      <c r="C37" s="5"/>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="9"/>
-      <c r="C38" s="5"/>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="9"/>
-      <c r="C39" s="5"/>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="9"/>
-      <c r="C40" s="5"/>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" s="9"/>
-      <c r="C41" s="5"/>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" s="9"/>
-      <c r="C42" s="5"/>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" s="9"/>
-      <c r="C43" s="5"/>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" s="9"/>
-      <c r="C44" s="5"/>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" s="9"/>
-      <c r="C45" s="5"/>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" s="9"/>
-      <c r="C46" s="5"/>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" s="9"/>
-      <c r="C47" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>